<commit_message>
Refactor application code and remove obsolete implementations
</commit_message>
<xml_diff>
--- a/outputs/worldo_collect_埋点计划.xlsx
+++ b/outputs/worldo_collect_埋点计划.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共字段" sheetId="1" r:id="R94e728a69e834d39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面访问统计" sheetId="2" r:id="R4dc86cec32b14e55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行为统计" sheetId="3" r:id="Rb826b08a1cd44431"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共字段" sheetId="1" r:id="R1a76944ab4014d33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面访问统计" sheetId="2" r:id="R7fd2accba71042b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行为统计" sheetId="3" r:id="R44edd473de7046e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -320,8 +320,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CommonFieldsTable" displayName="CommonFieldsTable" ref="A1:D12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:D12"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CommonFieldsTable" displayName="CommonFieldsTable" ref="A1:D16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:D16"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="位置"/>
     <x:tableColumn id="2" name="字段"/>
@@ -351,8 +351,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BehaviorStatsTable" displayName="BehaviorStatsTable" ref="A1:I27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I27"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BehaviorStatsTable" displayName="BehaviorStatsTable" ref="A1:I28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I28"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="统计"/>
     <x:tableColumn id="2" name="加入场景"/>
@@ -641,16 +641,16 @@
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="24" t="str">
-        <x:v>Body</x:v>
+        <x:v>Header</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>action_type</x:v>
+        <x:v>x-app-environment</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>pageview 或 event</x:v>
+        <x:v>production 或 test</x:v>
       </x:c>
       <x:c r="D6" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -658,10 +658,10 @@
         <x:v>Body</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>action</x:v>
+        <x:v>events</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
-        <x:v>页面名或事件名</x:v>
+        <x:v>本次从本地队列领取的事件数组，最多 500 条</x:v>
       </x:c>
       <x:c r="D7" s="25" t="str">
         <x:v>是</x:v>
@@ -672,13 +672,13 @@
         <x:v>Body</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>object1</x:v>
+        <x:v>events[].event_id</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str">
-        <x:v>业务对象 ID / query，按具体统计项传</x:v>
+        <x:v>客户端生成并在重试中保持不变的 UUID v4</x:v>
       </x:c>
       <x:c r="D8" s="25" t="str">
-        <x:v>是，非空才传</x:v>
+        <x:v>是</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -686,13 +686,13 @@
         <x:v>Body</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>object2</x:v>
+        <x:v>events[].action_type</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
-        <x:v>第二业务对象 ID / tickN，按具体统计项传</x:v>
+        <x:v>pageview、event 或 pay_event</x:v>
       </x:c>
       <x:c r="D9" s="25" t="str">
-        <x:v>是，非空才传</x:v>
+        <x:v>是</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
@@ -700,47 +700,103 @@
         <x:v>Body</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>object3</x:v>
+        <x:v>events[].action</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
-        <x:v>第三业务对象 ID，按具体统计项传</x:v>
+        <x:v>页面名或事件名</x:v>
       </x:c>
       <x:c r="D10" s="25" t="str">
-        <x:v>是，非空才传</x:v>
+        <x:v>是</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="24" t="str">
+        <x:v>Body</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>events[].app_timestamp</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>事件发生时的 Unix 毫秒时间戳</x:v>
+      </x:c>
+      <x:c r="D11" s="25" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="24" t="str">
+        <x:v>Body</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="str">
+        <x:v>events[].object1</x:v>
+      </x:c>
+      <x:c r="C12" s="16" t="str">
+        <x:v>业务对象 ID / query；无值传空字符串</x:v>
+      </x:c>
+      <x:c r="D12" s="25" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="24" t="str">
+        <x:v>Body</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="str">
+        <x:v>events[].object2</x:v>
+      </x:c>
+      <x:c r="C13" s="16" t="str">
+        <x:v>第二业务对象 ID / tickN；无值传空字符串</x:v>
+      </x:c>
+      <x:c r="D13" s="25" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="24" t="str">
+        <x:v>Body</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="str">
+        <x:v>events[].object3</x:v>
+      </x:c>
+      <x:c r="C14" s="16" t="str">
+        <x:v>第三业务对象 ID；无值传空字符串</x:v>
+      </x:c>
+      <x:c r="D14" s="25" t="str">
+        <x:v>是</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="24" t="str">
         <x:v>服务端</x:v>
       </x:c>
-      <x:c r="B11" s="16" t="str">
+      <x:c r="B15" s="16" t="str">
         <x:v>IP address</x:v>
       </x:c>
-      <x:c r="C11" s="16" t="str">
+      <x:c r="C15" s="16" t="str">
         <x:v>collect 服务端从请求来源 IP 获取</x:v>
       </x:c>
-      <x:c r="D11" s="25" t="str">
+      <x:c r="D15" s="25" t="str">
         <x:v>否</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="30" customHeight="1">
-      <x:c r="A12" s="26" t="str">
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="26" t="str">
         <x:v>服务端</x:v>
       </x:c>
-      <x:c r="B12" s="27" t="str">
+      <x:c r="B16" s="27" t="str">
         <x:v>created_at</x:v>
       </x:c>
-      <x:c r="C12" s="27" t="str">
+      <x:c r="C16" s="27" t="str">
         <x:v>collect 服务端生成</x:v>
       </x:c>
-      <x:c r="D12" s="28" t="str">
+      <x:c r="D16" s="28" t="str">
         <x:v>否</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45fc88f46461427c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14bd2793bc484c96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1405,7 +1461,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ff4c212c9b44c6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78ae1cec13e34987"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1456,10 +1512,10 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="24" t="str">
-        <x:v>create_worldo_submit_start</x:v>
+        <x:v>startup_first_report</x:v>
       </x:c>
       <x:c r="B2" s="16" t="str">
-        <x:v>点击 Create 后，调用 create 接口前</x:v>
+        <x:v>Collect recorder 准备完成后立即记录，早于 runApp 和 GenesisTelemetry.initialize()</x:v>
       </x:c>
       <x:c r="C2" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1468,21 +1524,21 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E2" s="16" t="str">
-        <x:v>create_worldo_submit_start</x:v>
+        <x:v>startup_first_report</x:v>
       </x:c>
       <x:c r="F2" s="16" t="str"/>
       <x:c r="G2" s="16" t="str"/>
       <x:c r="H2" s="16" t="str"/>
       <x:c r="I2" s="25" t="str">
-        <x:v>此时还没有 oid，不传 object1</x:v>
+        <x:v>main.runGenesisApp / AppStartupCoordinator</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="24" t="str">
-        <x:v>create_worldo_submit_success</x:v>
+        <x:v>create_worldo_submit_start</x:v>
       </x:c>
       <x:c r="B3" s="16" t="str">
-        <x:v>create 接口返回 oid 后</x:v>
+        <x:v>点击 Create 后，调用 create 接口前</x:v>
       </x:c>
       <x:c r="C3" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1491,23 +1547,21 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E3" s="16" t="str">
-        <x:v>create_worldo_submit_success</x:v>
-      </x:c>
-      <x:c r="F3" s="16" t="str">
-        <x:v>oid</x:v>
-      </x:c>
+        <x:v>create_worldo_submit_start</x:v>
+      </x:c>
+      <x:c r="F3" s="16" t="str"/>
       <x:c r="G3" s="16" t="str"/>
       <x:c r="H3" s="16" t="str"/>
       <x:c r="I3" s="25" t="str">
-        <x:v>CreateOriginResult.oid</x:v>
+        <x:v>此时还没有 oid，不传 object1</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="24" t="str">
-        <x:v>create_worldo_async_complete</x:v>
+        <x:v>create_worldo_submit_success</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>轮询 origin/info 确认完成后</x:v>
+        <x:v>create 接口返回 oid 后</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1516,7 +1570,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E4" s="16" t="str">
-        <x:v>create_worldo_async_complete</x:v>
+        <x:v>create_worldo_submit_success</x:v>
       </x:c>
       <x:c r="F4" s="16" t="str">
         <x:v>oid</x:v>
@@ -1524,15 +1578,15 @@
       <x:c r="G4" s="16" t="str"/>
       <x:c r="H4" s="16" t="str"/>
       <x:c r="I4" s="25" t="str">
-        <x:v>OriginPendingSubmissionCoordinator completed outcome</x:v>
+        <x:v>CreateOriginResult.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="24" t="str">
-        <x:v>edit_worldo_submit_start</x:v>
+        <x:v>create_worldo_async_complete</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
-        <x:v>点击 Publish 后，调用 update 接口前</x:v>
+        <x:v>轮询 origin/info 确认完成后</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1541,7 +1595,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
-        <x:v>edit_worldo_submit_start</x:v>
+        <x:v>create_worldo_async_complete</x:v>
       </x:c>
       <x:c r="F5" s="16" t="str">
         <x:v>oid</x:v>
@@ -1549,15 +1603,15 @@
       <x:c r="G5" s="16" t="str"/>
       <x:c r="H5" s="16" t="str"/>
       <x:c r="I5" s="25" t="str">
-        <x:v>EditOriginPage draft.basics.originId</x:v>
+        <x:v>OriginPendingSubmissionCoordinator completed outcome</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="24" t="str">
-        <x:v>edit_worldo_submit_success</x:v>
+        <x:v>edit_worldo_submit_start</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>update 接口返回成功后</x:v>
+        <x:v>点击 Publish 后，调用 update 接口前</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1566,7 +1620,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str">
-        <x:v>edit_worldo_submit_success</x:v>
+        <x:v>edit_worldo_submit_start</x:v>
       </x:c>
       <x:c r="F6" s="16" t="str">
         <x:v>oid</x:v>
@@ -1574,15 +1628,15 @@
       <x:c r="G6" s="16" t="str"/>
       <x:c r="H6" s="16" t="str"/>
       <x:c r="I6" s="25" t="str">
-        <x:v>CreateOriginResult.oid</x:v>
+        <x:v>EditOriginPage draft.basics.originId</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="24" t="str">
-        <x:v>edit_worldo_async_complete</x:v>
+        <x:v>edit_worldo_submit_success</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>轮询 origin/info 确认完成后</x:v>
+        <x:v>update 接口返回成功后</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1591,7 +1645,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E7" s="16" t="str">
-        <x:v>edit_worldo_async_complete</x:v>
+        <x:v>edit_worldo_submit_success</x:v>
       </x:c>
       <x:c r="F7" s="16" t="str">
         <x:v>oid</x:v>
@@ -1599,15 +1653,15 @@
       <x:c r="G7" s="16" t="str"/>
       <x:c r="H7" s="16" t="str"/>
       <x:c r="I7" s="25" t="str">
-        <x:v>OriginPendingSubmissionCoordinator completed outcome</x:v>
+        <x:v>CreateOriginResult.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="24" t="str">
-        <x:v>worldo_launch_submit_start</x:v>
+        <x:v>edit_worldo_async_complete</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>launch 确认提交，调用 origin/launch 前</x:v>
+        <x:v>轮询 origin/info 确认完成后</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1616,7 +1670,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str">
-        <x:v>worldo_launch_submit_start</x:v>
+        <x:v>edit_worldo_async_complete</x:v>
       </x:c>
       <x:c r="F8" s="16" t="str">
         <x:v>oid</x:v>
@@ -1624,15 +1678,15 @@
       <x:c r="G8" s="16" t="str"/>
       <x:c r="H8" s="16" t="str"/>
       <x:c r="I8" s="25" t="str">
-        <x:v>OriginDetail.oid</x:v>
+        <x:v>OriginPendingSubmissionCoordinator completed outcome</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
       <x:c r="A9" s="24" t="str">
-        <x:v>worldo_launch_submit_success</x:v>
+        <x:v>worldo_launch_submit_start</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>origin/launch 返回 wid 后</x:v>
+        <x:v>launch 确认提交，调用 origin/launch 前</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1641,25 +1695,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
-        <x:v>worldo_launch_submit_success</x:v>
+        <x:v>worldo_launch_submit_start</x:v>
       </x:c>
       <x:c r="F9" s="16" t="str">
         <x:v>oid</x:v>
       </x:c>
-      <x:c r="G9" s="16" t="str">
-        <x:v>wid</x:v>
-      </x:c>
+      <x:c r="G9" s="16" t="str"/>
       <x:c r="H9" s="16" t="str"/>
       <x:c r="I9" s="25" t="str">
-        <x:v>OriginDetail.oid；origin/launch 返回 world_id/wid</x:v>
+        <x:v>OriginDetail.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
       <x:c r="A10" s="24" t="str">
-        <x:v>worldo_launch_async_complete</x:v>
+        <x:v>worldo_launch_submit_success</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>轮询确认 tick1 完成后</x:v>
+        <x:v>origin/launch 返回 wid 后</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1668,7 +1720,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
-        <x:v>worldo_launch_async_complete</x:v>
+        <x:v>worldo_launch_submit_success</x:v>
       </x:c>
       <x:c r="F10" s="16" t="str">
         <x:v>oid</x:v>
@@ -1678,15 +1730,15 @@
       </x:c>
       <x:c r="H10" s="16" t="str"/>
       <x:c r="I10" s="25" t="str">
-        <x:v>OriginLaunchCoordinator completed outcome</x:v>
+        <x:v>OriginDetail.oid；origin/launch 返回 world_id/wid</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="24" t="str">
-        <x:v>world_progress_submit_start</x:v>
+        <x:v>worldo_launch_async_complete</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>点击 Progress 后，调用 world/tick 前</x:v>
+        <x:v>轮询确认 tick1 完成后</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1695,23 +1747,25 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str">
-        <x:v>world_progress_submit_start</x:v>
+        <x:v>worldo_launch_async_complete</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
+        <x:v>oid</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G11" s="16" t="str"/>
       <x:c r="H11" s="16" t="str"/>
       <x:c r="I11" s="25" t="str">
-        <x:v>WorldPage.widget.wid</x:v>
+        <x:v>OriginLaunchCoordinator completed outcome</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="24" t="str">
-        <x:v>world_progress_submit_success</x:v>
+        <x:v>world_progress_submit_start</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
-        <x:v>world/tick 返回成功后</x:v>
+        <x:v>点击 Progress 后，调用 world/tick 前</x:v>
       </x:c>
       <x:c r="C12" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1720,25 +1774,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
-        <x:v>world_progress_submit_success</x:v>
+        <x:v>world_progress_submit_start</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G12" s="16" t="str">
-        <x:v>tickN</x:v>
-      </x:c>
+      <x:c r="G12" s="16" t="str"/>
       <x:c r="H12" s="16" t="str"/>
       <x:c r="I12" s="25" t="str">
-        <x:v>WorldPage.widget.wid；world/tick 返回 tick_cnt</x:v>
+        <x:v>WorldPage.widget.wid</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="24" t="str">
-        <x:v>world_progress_async_complete</x:v>
+        <x:v>world_progress_submit_success</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
-        <x:v>world/info 轮询确认不再 progressing 后</x:v>
+        <x:v>world/tick 返回成功后</x:v>
       </x:c>
       <x:c r="C13" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1747,7 +1799,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
-        <x:v>world_progress_async_complete</x:v>
+        <x:v>world_progress_submit_success</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
         <x:v>wid</x:v>
@@ -1757,15 +1809,15 @@
       </x:c>
       <x:c r="H13" s="16" t="str"/>
       <x:c r="I13" s="25" t="str">
-        <x:v>WorldPage.widget.wid；刷新后的 WorldDetail.tickCount</x:v>
+        <x:v>WorldPage.widget.wid；world/tick 返回 tick_cnt</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="24" t="str">
-        <x:v>login</x:v>
+        <x:v>world_progress_async_complete</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
-        <x:v>登录成功写入用户态后</x:v>
+        <x:v>world/info 轮询确认不再 progressing 后</x:v>
       </x:c>
       <x:c r="C14" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1774,21 +1826,25 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
-        <x:v>login</x:v>
-      </x:c>
-      <x:c r="F14" s="16" t="str"/>
-      <x:c r="G14" s="16" t="str"/>
+        <x:v>world_progress_async_complete</x:v>
+      </x:c>
+      <x:c r="F14" s="16" t="str">
+        <x:v>wid</x:v>
+      </x:c>
+      <x:c r="G14" s="16" t="str">
+        <x:v>tickN</x:v>
+      </x:c>
       <x:c r="H14" s="16" t="str"/>
       <x:c r="I14" s="25" t="str">
-        <x:v>BackendAuthCoordinator login success</x:v>
+        <x:v>WorldPage.widget.wid；刷新后的 WorldDetail.tickCount</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="24" t="str">
-        <x:v>logout</x:v>
+        <x:v>login</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
-        <x:v>logout 清理用户态前</x:v>
+        <x:v>登录成功写入用户态后</x:v>
       </x:c>
       <x:c r="C15" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1797,21 +1853,21 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
-        <x:v>logout</x:v>
+        <x:v>login</x:v>
       </x:c>
       <x:c r="F15" s="16" t="str"/>
       <x:c r="G15" s="16" t="str"/>
       <x:c r="H15" s="16" t="str"/>
       <x:c r="I15" s="25" t="str">
-        <x:v>BackendAuthCoordinator signOut</x:v>
+        <x:v>BackendAuthCoordinator login success</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="24" t="str">
-        <x:v>delete_account</x:v>
+        <x:v>logout</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
-        <x:v>删除账号成功后</x:v>
+        <x:v>logout 清理用户态前</x:v>
       </x:c>
       <x:c r="C16" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1820,21 +1876,21 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E16" s="16" t="str">
-        <x:v>delete_account</x:v>
+        <x:v>logout</x:v>
       </x:c>
       <x:c r="F16" s="16" t="str"/>
       <x:c r="G16" s="16" t="str"/>
       <x:c r="H16" s="16" t="str"/>
       <x:c r="I16" s="25" t="str">
-        <x:v>BackendAuthCoordinator deleteAccount</x:v>
+        <x:v>BackendAuthCoordinator signOut</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>request_submit</x:v>
+        <x:v>delete_account</x:v>
       </x:c>
       <x:c r="B17" s="16" t="str">
-        <x:v>world request 提交成功后</x:v>
+        <x:v>删除账号成功后</x:v>
       </x:c>
       <x:c r="C17" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1843,23 +1899,21 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E17" s="16" t="str">
-        <x:v>request_submit</x:v>
-      </x:c>
-      <x:c r="F17" s="16" t="str">
-        <x:v>wid</x:v>
-      </x:c>
+        <x:v>delete_account</x:v>
+      </x:c>
+      <x:c r="F17" s="16" t="str"/>
       <x:c r="G17" s="16" t="str"/>
       <x:c r="H17" s="16" t="str"/>
       <x:c r="I17" s="25" t="str">
-        <x:v>WorldPage.widget.wid</x:v>
+        <x:v>BackendAuthCoordinator deleteAccount</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>search_click</x:v>
+        <x:v>request_submit</x:v>
       </x:c>
       <x:c r="B18" s="16" t="str">
-        <x:v>点击搜索结果</x:v>
+        <x:v>world request 提交成功后</x:v>
       </x:c>
       <x:c r="C18" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1868,25 +1922,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E18" s="16" t="str">
-        <x:v>search_click</x:v>
+        <x:v>request_submit</x:v>
       </x:c>
       <x:c r="F18" s="16" t="str">
-        <x:v>query</x:v>
-      </x:c>
-      <x:c r="G18" s="16" t="str">
-        <x:v>oid/wid/uid</x:v>
-      </x:c>
+        <x:v>wid</x:v>
+      </x:c>
+      <x:c r="G18" s="16" t="str"/>
       <x:c r="H18" s="16" t="str"/>
       <x:c r="I18" s="25" t="str">
-        <x:v>SearchPage._activeQuery；SearchResultItem.entityId</x:v>
+        <x:v>WorldPage.widget.wid</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
       <x:c r="A19" s="24" t="str">
-        <x:v>home_my_worlds_click</x:v>
+        <x:v>search_click</x:v>
       </x:c>
       <x:c r="B19" s="16" t="str">
-        <x:v>点击 My worlds item</x:v>
+        <x:v>点击搜索结果</x:v>
       </x:c>
       <x:c r="C19" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1895,23 +1947,25 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E19" s="16" t="str">
-        <x:v>home_my_worlds_click</x:v>
+        <x:v>search_click</x:v>
       </x:c>
       <x:c r="F19" s="16" t="str">
-        <x:v>wid</x:v>
-      </x:c>
-      <x:c r="G19" s="16" t="str"/>
+        <x:v>query</x:v>
+      </x:c>
+      <x:c r="G19" s="16" t="str">
+        <x:v>oid/wid/uid</x:v>
+      </x:c>
       <x:c r="H19" s="16" t="str"/>
       <x:c r="I19" s="25" t="str">
-        <x:v>WorldListItem.wid</x:v>
+        <x:v>SearchPage._activeQuery；SearchResultItem.entityId</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
       <x:c r="A20" s="24" t="str">
-        <x:v>home_popular_click</x:v>
+        <x:v>home_my_worlds_click</x:v>
       </x:c>
       <x:c r="B20" s="16" t="str">
-        <x:v>点击 Popular item</x:v>
+        <x:v>点击 My worlds item</x:v>
       </x:c>
       <x:c r="C20" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1920,23 +1974,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E20" s="16" t="str">
-        <x:v>home_popular_click</x:v>
+        <x:v>home_my_worlds_click</x:v>
       </x:c>
       <x:c r="F20" s="16" t="str">
-        <x:v>oid</x:v>
+        <x:v>wid</x:v>
       </x:c>
       <x:c r="G20" s="16" t="str"/>
       <x:c r="H20" s="16" t="str"/>
       <x:c r="I20" s="25" t="str">
-        <x:v>OriginListItem.oid</x:v>
+        <x:v>WorldListItem.wid</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
       <x:c r="A21" s="24" t="str">
-        <x:v>worldo_list_click</x:v>
+        <x:v>home_popular_click</x:v>
       </x:c>
       <x:c r="B21" s="16" t="str">
-        <x:v>点击 worldo list item</x:v>
+        <x:v>点击 Popular item</x:v>
       </x:c>
       <x:c r="C21" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1945,7 +1999,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E21" s="16" t="str">
-        <x:v>worldo_list_click</x:v>
+        <x:v>home_popular_click</x:v>
       </x:c>
       <x:c r="F21" s="16" t="str">
         <x:v>oid</x:v>
@@ -1958,10 +2012,10 @@
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="24" t="str">
-        <x:v>me_click</x:v>
+        <x:v>worldo_list_click</x:v>
       </x:c>
       <x:c r="B22" s="16" t="str">
-        <x:v>点击 Me/Profile 页面 oid/wid 内容</x:v>
+        <x:v>点击 worldo list item</x:v>
       </x:c>
       <x:c r="C22" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1970,23 +2024,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E22" s="16" t="str">
-        <x:v>me_click</x:v>
+        <x:v>worldo_list_click</x:v>
       </x:c>
       <x:c r="F22" s="16" t="str">
-        <x:v>oid/wid</x:v>
+        <x:v>oid</x:v>
       </x:c>
       <x:c r="G22" s="16" t="str"/>
       <x:c r="H22" s="16" t="str"/>
       <x:c r="I22" s="25" t="str">
-        <x:v>UserProfileOriginItem.oid 或 UserProfileWorldItem.wid</x:v>
+        <x:v>OriginListItem.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
       <x:c r="A23" s="24" t="str">
-        <x:v>worldo_map_click</x:v>
+        <x:v>me_click</x:v>
       </x:c>
       <x:c r="B23" s="16" t="str">
-        <x:v>点击 worldo map 任意位置</x:v>
+        <x:v>点击 Me/Profile 页面 oid/wid 内容</x:v>
       </x:c>
       <x:c r="C23" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1995,23 +2049,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E23" s="16" t="str">
-        <x:v>worldo_map_click</x:v>
+        <x:v>me_click</x:v>
       </x:c>
       <x:c r="F23" s="16" t="str">
-        <x:v>oid</x:v>
+        <x:v>oid/wid</x:v>
       </x:c>
       <x:c r="G23" s="16" t="str"/>
       <x:c r="H23" s="16" t="str"/>
       <x:c r="I23" s="25" t="str">
-        <x:v>OriginDetail.oid</x:v>
+        <x:v>UserProfileOriginItem.oid 或 UserProfileWorldItem.wid</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
       <x:c r="A24" s="24" t="str">
-        <x:v>world_locations_click</x:v>
+        <x:v>worldo_map_click</x:v>
       </x:c>
       <x:c r="B24" s="16" t="str">
-        <x:v>点击 location 列表项</x:v>
+        <x:v>点击 worldo map 任意位置</x:v>
       </x:c>
       <x:c r="C24" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2020,25 +2074,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E24" s="16" t="str">
-        <x:v>world_locations_click</x:v>
+        <x:v>worldo_map_click</x:v>
       </x:c>
       <x:c r="F24" s="16" t="str">
-        <x:v>wid</x:v>
-      </x:c>
-      <x:c r="G24" s="16" t="str">
-        <x:v>loc_id</x:v>
-      </x:c>
+        <x:v>oid</x:v>
+      </x:c>
+      <x:c r="G24" s="16" t="str"/>
       <x:c r="H24" s="16" t="str"/>
       <x:c r="I24" s="25" t="str">
-        <x:v>WorldDetail.worldId；WorldPoint sceneId/pointId/id</x:v>
+        <x:v>OriginDetail.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="24" t="str">
-        <x:v>world_map_click</x:v>
+        <x:v>world_locations_click</x:v>
       </x:c>
       <x:c r="B25" s="16" t="str">
-        <x:v>点击 world map 任意位置</x:v>
+        <x:v>点击 location 列表项</x:v>
       </x:c>
       <x:c r="C25" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2047,23 +2099,25 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E25" s="16" t="str">
-        <x:v>world_map_click</x:v>
+        <x:v>world_locations_click</x:v>
       </x:c>
       <x:c r="F25" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G25" s="16" t="str"/>
+      <x:c r="G25" s="16" t="str">
+        <x:v>loc_id</x:v>
+      </x:c>
       <x:c r="H25" s="16" t="str"/>
       <x:c r="I25" s="25" t="str">
-        <x:v>WorldPage.widget.wid</x:v>
+        <x:v>WorldDetail.worldId；WorldPoint sceneId/pointId/id</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="24" t="str">
-        <x:v>location_chat_send_message</x:v>
+        <x:v>world_map_click</x:v>
       </x:c>
       <x:c r="B26" s="16" t="str">
-        <x:v>location chat 发消息成功后</x:v>
+        <x:v>点击 world map 任意位置</x:v>
       </x:c>
       <x:c r="C26" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2072,52 +2126,77 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E26" s="16" t="str">
-        <x:v>location_chat_send_message</x:v>
+        <x:v>world_map_click</x:v>
       </x:c>
       <x:c r="F26" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G26" s="16" t="str">
+      <x:c r="G26" s="16" t="str"/>
+      <x:c r="H26" s="16" t="str"/>
+      <x:c r="I26" s="25" t="str">
+        <x:v>WorldPage.widget.wid</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="A27" s="24" t="str">
+        <x:v>location_chat_send_message</x:v>
+      </x:c>
+      <x:c r="B27" s="16" t="str">
+        <x:v>location chat 发消息成功后</x:v>
+      </x:c>
+      <x:c r="C27" s="16" t="str">
+        <x:v>GenesisTelemetry.collectLog</x:v>
+      </x:c>
+      <x:c r="D27" s="16" t="str">
+        <x:v>event</x:v>
+      </x:c>
+      <x:c r="E27" s="16" t="str">
+        <x:v>location_chat_send_message</x:v>
+      </x:c>
+      <x:c r="F27" s="16" t="str">
+        <x:v>wid</x:v>
+      </x:c>
+      <x:c r="G27" s="16" t="str">
         <x:v>loc_id</x:v>
       </x:c>
-      <x:c r="H26" s="16" t="str">
+      <x:c r="H27" s="16" t="str">
         <x:v>message_id</x:v>
       </x:c>
-      <x:c r="I26" s="25" t="str">
+      <x:c r="I27" s="25" t="str">
         <x:v>LocationChatPage.widget.worldId；widget.locationId；ack.messageId</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="26" t="str">
+    <x:row r="28" ht="30" customHeight="1">
+      <x:c r="A28" s="26" t="str">
         <x:v>private_chat_send_message</x:v>
       </x:c>
-      <x:c r="B27" s="27" t="str">
+      <x:c r="B28" s="27" t="str">
         <x:v>私聊发送成功后</x:v>
       </x:c>
-      <x:c r="C27" s="27" t="str">
-        <x:v>GenesisTelemetry.collectLog</x:v>
-      </x:c>
-      <x:c r="D27" s="27" t="str">
-        <x:v>event</x:v>
-      </x:c>
-      <x:c r="E27" s="27" t="str">
+      <x:c r="C28" s="27" t="str">
+        <x:v>GenesisTelemetry.collectLog</x:v>
+      </x:c>
+      <x:c r="D28" s="27" t="str">
+        <x:v>event</x:v>
+      </x:c>
+      <x:c r="E28" s="27" t="str">
         <x:v>private_chat_send_message</x:v>
       </x:c>
-      <x:c r="F27" s="27" t="str">
+      <x:c r="F28" s="27" t="str">
         <x:v>peer_uid</x:v>
       </x:c>
-      <x:c r="G27" s="27" t="str">
+      <x:c r="G28" s="27" t="str">
         <x:v>message_id</x:v>
       </x:c>
-      <x:c r="H27" s="27" t="str"/>
-      <x:c r="I27" s="28" t="str">
+      <x:c r="H28" s="27" t="str"/>
+      <x:c r="I28" s="28" t="str">
         <x:v>ChatPage._peerUid；dm send 返回 message_id/id</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6904daa08c074bf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf0578f706e94998"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine Origin V2 flows and chat image handling
</commit_message>
<xml_diff>
--- a/outputs/worldo_collect_埋点计划.xlsx
+++ b/outputs/worldo_collect_埋点计划.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共字段" sheetId="1" r:id="R1a76944ab4014d33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面访问统计" sheetId="2" r:id="R7fd2accba71042b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行为统计" sheetId="3" r:id="R44edd473de7046e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共字段" sheetId="1" r:id="Rcf1d1f9bd36a47c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面访问统计" sheetId="2" r:id="Rd52b68d2d1874465"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行为统计" sheetId="3" r:id="Rdbe345f0a4be47f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -351,8 +351,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BehaviorStatsTable" displayName="BehaviorStatsTable" ref="A1:I28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I28"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BehaviorStatsTable" displayName="BehaviorStatsTable" ref="A1:I30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I30"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="统计"/>
     <x:tableColumn id="2" name="加入场景"/>
@@ -796,7 +796,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14bd2793bc484c96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfade454e388746b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1461,7 +1461,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78ae1cec13e34987"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36787318ecec4194"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2065,7 +2065,7 @@
         <x:v>worldo_map_click</x:v>
       </x:c>
       <x:c r="B24" s="16" t="str">
-        <x:v>点击 worldo map 任意位置</x:v>
+        <x:v>点击旧版 worldo map 任意位置</x:v>
       </x:c>
       <x:c r="C24" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2087,10 +2087,10 @@
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="24" t="str">
-        <x:v>world_locations_click</x:v>
+        <x:v>worldo_tilemap_click</x:v>
       </x:c>
       <x:c r="B25" s="16" t="str">
-        <x:v>点击 location 列表项</x:v>
+        <x:v>点击 Tilemap 版 worldo map 任意位置</x:v>
       </x:c>
       <x:c r="C25" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2099,25 +2099,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E25" s="16" t="str">
-        <x:v>world_locations_click</x:v>
+        <x:v>worldo_tilemap_click</x:v>
       </x:c>
       <x:c r="F25" s="16" t="str">
-        <x:v>wid</x:v>
-      </x:c>
-      <x:c r="G25" s="16" t="str">
-        <x:v>loc_id</x:v>
-      </x:c>
+        <x:v>oid</x:v>
+      </x:c>
+      <x:c r="G25" s="16" t="str"/>
       <x:c r="H25" s="16" t="str"/>
       <x:c r="I25" s="25" t="str">
-        <x:v>WorldDetail.worldId；WorldPoint sceneId/pointId/id</x:v>
+        <x:v>OriginDetail.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="24" t="str">
-        <x:v>world_map_click</x:v>
+        <x:v>world_locations_click</x:v>
       </x:c>
       <x:c r="B26" s="16" t="str">
-        <x:v>点击 world map 任意位置</x:v>
+        <x:v>点击 location 列表项</x:v>
       </x:c>
       <x:c r="C26" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2126,23 +2124,25 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E26" s="16" t="str">
-        <x:v>world_map_click</x:v>
+        <x:v>world_locations_click</x:v>
       </x:c>
       <x:c r="F26" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G26" s="16" t="str"/>
+      <x:c r="G26" s="16" t="str">
+        <x:v>loc_id</x:v>
+      </x:c>
       <x:c r="H26" s="16" t="str"/>
       <x:c r="I26" s="25" t="str">
-        <x:v>WorldPage.widget.wid</x:v>
+        <x:v>WorldDetail.worldId；WorldPoint sceneId/pointId/id</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
       <x:c r="A27" s="24" t="str">
-        <x:v>location_chat_send_message</x:v>
+        <x:v>world_map_click</x:v>
       </x:c>
       <x:c r="B27" s="16" t="str">
-        <x:v>location chat 发消息成功后</x:v>
+        <x:v>点击旧版 world map 任意位置</x:v>
       </x:c>
       <x:c r="C27" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2151,52 +2151,102 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E27" s="16" t="str">
-        <x:v>location_chat_send_message</x:v>
+        <x:v>world_map_click</x:v>
       </x:c>
       <x:c r="F27" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G27" s="16" t="str">
+      <x:c r="G27" s="16" t="str"/>
+      <x:c r="H27" s="16" t="str"/>
+      <x:c r="I27" s="25" t="str">
+        <x:v>WorldPage.widget.wid</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="30" customHeight="1">
+      <x:c r="A28" s="24" t="str">
+        <x:v>world_tilemap_click</x:v>
+      </x:c>
+      <x:c r="B28" s="16" t="str">
+        <x:v>点击 Tilemap 版 world map 任意位置</x:v>
+      </x:c>
+      <x:c r="C28" s="16" t="str">
+        <x:v>GenesisTelemetry.collectLog</x:v>
+      </x:c>
+      <x:c r="D28" s="16" t="str">
+        <x:v>event</x:v>
+      </x:c>
+      <x:c r="E28" s="16" t="str">
+        <x:v>world_tilemap_click</x:v>
+      </x:c>
+      <x:c r="F28" s="16" t="str">
+        <x:v>wid</x:v>
+      </x:c>
+      <x:c r="G28" s="16" t="str"/>
+      <x:c r="H28" s="16" t="str"/>
+      <x:c r="I28" s="25" t="str">
+        <x:v>WorldPage.widget.wid</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="30" customHeight="1">
+      <x:c r="A29" s="24" t="str">
+        <x:v>location_chat_send_message</x:v>
+      </x:c>
+      <x:c r="B29" s="16" t="str">
+        <x:v>location chat 发消息成功后</x:v>
+      </x:c>
+      <x:c r="C29" s="16" t="str">
+        <x:v>GenesisTelemetry.collectLog</x:v>
+      </x:c>
+      <x:c r="D29" s="16" t="str">
+        <x:v>event</x:v>
+      </x:c>
+      <x:c r="E29" s="16" t="str">
+        <x:v>location_chat_send_message</x:v>
+      </x:c>
+      <x:c r="F29" s="16" t="str">
+        <x:v>wid</x:v>
+      </x:c>
+      <x:c r="G29" s="16" t="str">
         <x:v>loc_id</x:v>
       </x:c>
-      <x:c r="H27" s="16" t="str">
+      <x:c r="H29" s="16" t="str">
         <x:v>message_id</x:v>
       </x:c>
-      <x:c r="I27" s="25" t="str">
+      <x:c r="I29" s="25" t="str">
         <x:v>LocationChatPage.widget.worldId；widget.locationId；ack.messageId</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="30" customHeight="1">
-      <x:c r="A28" s="26" t="str">
+    <x:row r="30" ht="30" customHeight="1">
+      <x:c r="A30" s="26" t="str">
         <x:v>private_chat_send_message</x:v>
       </x:c>
-      <x:c r="B28" s="27" t="str">
+      <x:c r="B30" s="27" t="str">
         <x:v>私聊发送成功后</x:v>
       </x:c>
-      <x:c r="C28" s="27" t="str">
-        <x:v>GenesisTelemetry.collectLog</x:v>
-      </x:c>
-      <x:c r="D28" s="27" t="str">
-        <x:v>event</x:v>
-      </x:c>
-      <x:c r="E28" s="27" t="str">
+      <x:c r="C30" s="27" t="str">
+        <x:v>GenesisTelemetry.collectLog</x:v>
+      </x:c>
+      <x:c r="D30" s="27" t="str">
+        <x:v>event</x:v>
+      </x:c>
+      <x:c r="E30" s="27" t="str">
         <x:v>private_chat_send_message</x:v>
       </x:c>
-      <x:c r="F28" s="27" t="str">
+      <x:c r="F30" s="27" t="str">
         <x:v>peer_uid</x:v>
       </x:c>
-      <x:c r="G28" s="27" t="str">
+      <x:c r="G30" s="27" t="str">
         <x:v>message_id</x:v>
       </x:c>
-      <x:c r="H28" s="27" t="str"/>
-      <x:c r="I28" s="28" t="str">
+      <x:c r="H30" s="27" t="str"/>
+      <x:c r="I30" s="28" t="str">
         <x:v>ChatPage._peerUid；dm send 返回 message_id/id</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf0578f706e94998"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R731b57d7abd54656"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine application flows and supporting data handling
</commit_message>
<xml_diff>
--- a/outputs/worldo_collect_埋点计划.xlsx
+++ b/outputs/worldo_collect_埋点计划.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共字段" sheetId="1" r:id="Rcf1d1f9bd36a47c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面访问统计" sheetId="2" r:id="Rd52b68d2d1874465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行为统计" sheetId="3" r:id="Rdbe345f0a4be47f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共字段" sheetId="1" r:id="Ra62d3ab2547242e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面访问统计" sheetId="2" r:id="R336be141075a421b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行为统计" sheetId="3" r:id="Re0d17c05e75543f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -351,8 +351,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BehaviorStatsTable" displayName="BehaviorStatsTable" ref="A1:I30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I30"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BehaviorStatsTable" displayName="BehaviorStatsTable" ref="A1:I31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I31"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="统计"/>
     <x:tableColumn id="2" name="加入场景"/>
@@ -796,7 +796,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfade454e388746b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3c5215d210e4d57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1461,7 +1461,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36787318ecec4194"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f9496541214570"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1683,10 +1683,10 @@
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
       <x:c r="A9" s="24" t="str">
-        <x:v>worldo_launch_submit_start</x:v>
+        <x:v>worldo_launch_opening</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>launch 确认提交，调用 origin/launch 前</x:v>
+        <x:v>从 Opening 模块角色头像的 Select to launch 开启 launch</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1695,7 +1695,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
-        <x:v>worldo_launch_submit_start</x:v>
+        <x:v>worldo_launch_opening</x:v>
       </x:c>
       <x:c r="F9" s="16" t="str">
         <x:v>oid</x:v>
@@ -1703,15 +1703,15 @@
       <x:c r="G9" s="16" t="str"/>
       <x:c r="H9" s="16" t="str"/>
       <x:c r="I9" s="25" t="str">
-        <x:v>OriginDetail.oid</x:v>
+        <x:v>OriginWorldPage._selectAndLaunchPresetRole；OriginDetail.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
       <x:c r="A10" s="24" t="str">
-        <x:v>worldo_launch_submit_success</x:v>
+        <x:v>worldo_launch_sheet</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>origin/launch 返回 wid 后</x:v>
+        <x:v>从 Setup Your Role sheet 确认开启 launch</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1720,25 +1720,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
-        <x:v>worldo_launch_submit_success</x:v>
+        <x:v>worldo_launch_sheet</x:v>
       </x:c>
       <x:c r="F10" s="16" t="str">
         <x:v>oid</x:v>
       </x:c>
-      <x:c r="G10" s="16" t="str">
-        <x:v>wid</x:v>
-      </x:c>
+      <x:c r="G10" s="16" t="str"/>
       <x:c r="H10" s="16" t="str"/>
       <x:c r="I10" s="25" t="str">
-        <x:v>OriginDetail.oid；origin/launch 返回 world_id/wid</x:v>
+        <x:v>OriginWorldPage._openLaunchRoleSheet；OriginDetail.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="24" t="str">
-        <x:v>worldo_launch_async_complete</x:v>
+        <x:v>worldo_launch_submit_success</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>轮询确认 tick1 完成后</x:v>
+        <x:v>origin/launch 返回 wid 后</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1747,7 +1745,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str">
-        <x:v>worldo_launch_async_complete</x:v>
+        <x:v>worldo_launch_submit_success</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
         <x:v>oid</x:v>
@@ -1757,15 +1755,15 @@
       </x:c>
       <x:c r="H11" s="16" t="str"/>
       <x:c r="I11" s="25" t="str">
-        <x:v>OriginLaunchCoordinator completed outcome</x:v>
+        <x:v>OriginDetail.oid；origin/launch 返回 world_id/wid</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="24" t="str">
-        <x:v>world_progress_submit_start</x:v>
+        <x:v>worldo_launch_async_complete</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
-        <x:v>点击 Progress 后，调用 world/tick 前</x:v>
+        <x:v>轮询确认 tick1 完成后</x:v>
       </x:c>
       <x:c r="C12" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1774,23 +1772,25 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
-        <x:v>world_progress_submit_start</x:v>
+        <x:v>worldo_launch_async_complete</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
+        <x:v>oid</x:v>
+      </x:c>
+      <x:c r="G12" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G12" s="16" t="str"/>
       <x:c r="H12" s="16" t="str"/>
       <x:c r="I12" s="25" t="str">
-        <x:v>WorldPage.widget.wid</x:v>
+        <x:v>OriginLaunchCoordinator completed outcome</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="24" t="str">
-        <x:v>world_progress_submit_success</x:v>
+        <x:v>world_progress_submit_start</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
-        <x:v>world/tick 返回成功后</x:v>
+        <x:v>点击 Progress 后，调用 world/tick 前</x:v>
       </x:c>
       <x:c r="C13" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1799,25 +1799,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
-        <x:v>world_progress_submit_success</x:v>
+        <x:v>world_progress_submit_start</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G13" s="16" t="str">
-        <x:v>tickN</x:v>
-      </x:c>
+      <x:c r="G13" s="16" t="str"/>
       <x:c r="H13" s="16" t="str"/>
       <x:c r="I13" s="25" t="str">
-        <x:v>WorldPage.widget.wid；world/tick 返回 tick_cnt</x:v>
+        <x:v>WorldPage.widget.wid</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="24" t="str">
-        <x:v>world_progress_async_complete</x:v>
+        <x:v>world_progress_submit_success</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
-        <x:v>world/info 轮询确认不再 progressing 后</x:v>
+        <x:v>world/tick 返回成功后</x:v>
       </x:c>
       <x:c r="C14" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1826,7 +1824,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
-        <x:v>world_progress_async_complete</x:v>
+        <x:v>world_progress_submit_success</x:v>
       </x:c>
       <x:c r="F14" s="16" t="str">
         <x:v>wid</x:v>
@@ -1836,15 +1834,15 @@
       </x:c>
       <x:c r="H14" s="16" t="str"/>
       <x:c r="I14" s="25" t="str">
-        <x:v>WorldPage.widget.wid；刷新后的 WorldDetail.tickCount</x:v>
+        <x:v>WorldPage.widget.wid；world/tick 返回 tick_cnt</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="24" t="str">
-        <x:v>login</x:v>
+        <x:v>world_progress_async_complete</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
-        <x:v>登录成功写入用户态后</x:v>
+        <x:v>world/info 轮询确认不再 progressing 后</x:v>
       </x:c>
       <x:c r="C15" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1853,21 +1851,25 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
-        <x:v>login</x:v>
-      </x:c>
-      <x:c r="F15" s="16" t="str"/>
-      <x:c r="G15" s="16" t="str"/>
+        <x:v>world_progress_async_complete</x:v>
+      </x:c>
+      <x:c r="F15" s="16" t="str">
+        <x:v>wid</x:v>
+      </x:c>
+      <x:c r="G15" s="16" t="str">
+        <x:v>tickN</x:v>
+      </x:c>
       <x:c r="H15" s="16" t="str"/>
       <x:c r="I15" s="25" t="str">
-        <x:v>BackendAuthCoordinator login success</x:v>
+        <x:v>WorldPage.widget.wid；刷新后的 WorldDetail.tickCount</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="24" t="str">
-        <x:v>logout</x:v>
+        <x:v>login</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
-        <x:v>logout 清理用户态前</x:v>
+        <x:v>登录成功写入用户态后</x:v>
       </x:c>
       <x:c r="C16" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1876,21 +1878,21 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E16" s="16" t="str">
-        <x:v>logout</x:v>
+        <x:v>login</x:v>
       </x:c>
       <x:c r="F16" s="16" t="str"/>
       <x:c r="G16" s="16" t="str"/>
       <x:c r="H16" s="16" t="str"/>
       <x:c r="I16" s="25" t="str">
-        <x:v>BackendAuthCoordinator signOut</x:v>
+        <x:v>BackendAuthCoordinator login success</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>delete_account</x:v>
+        <x:v>logout</x:v>
       </x:c>
       <x:c r="B17" s="16" t="str">
-        <x:v>删除账号成功后</x:v>
+        <x:v>logout 清理用户态前</x:v>
       </x:c>
       <x:c r="C17" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1899,21 +1901,21 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E17" s="16" t="str">
-        <x:v>delete_account</x:v>
+        <x:v>logout</x:v>
       </x:c>
       <x:c r="F17" s="16" t="str"/>
       <x:c r="G17" s="16" t="str"/>
       <x:c r="H17" s="16" t="str"/>
       <x:c r="I17" s="25" t="str">
-        <x:v>BackendAuthCoordinator deleteAccount</x:v>
+        <x:v>BackendAuthCoordinator signOut</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>request_submit</x:v>
+        <x:v>delete_account</x:v>
       </x:c>
       <x:c r="B18" s="16" t="str">
-        <x:v>world request 提交成功后</x:v>
+        <x:v>删除账号成功后</x:v>
       </x:c>
       <x:c r="C18" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1922,23 +1924,21 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E18" s="16" t="str">
-        <x:v>request_submit</x:v>
-      </x:c>
-      <x:c r="F18" s="16" t="str">
-        <x:v>wid</x:v>
-      </x:c>
+        <x:v>delete_account</x:v>
+      </x:c>
+      <x:c r="F18" s="16" t="str"/>
       <x:c r="G18" s="16" t="str"/>
       <x:c r="H18" s="16" t="str"/>
       <x:c r="I18" s="25" t="str">
-        <x:v>WorldPage.widget.wid</x:v>
+        <x:v>BackendAuthCoordinator deleteAccount</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
       <x:c r="A19" s="24" t="str">
-        <x:v>search_click</x:v>
+        <x:v>request_submit</x:v>
       </x:c>
       <x:c r="B19" s="16" t="str">
-        <x:v>点击搜索结果</x:v>
+        <x:v>world request 提交成功后</x:v>
       </x:c>
       <x:c r="C19" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1947,25 +1947,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E19" s="16" t="str">
-        <x:v>search_click</x:v>
+        <x:v>request_submit</x:v>
       </x:c>
       <x:c r="F19" s="16" t="str">
-        <x:v>query</x:v>
-      </x:c>
-      <x:c r="G19" s="16" t="str">
-        <x:v>oid/wid/uid</x:v>
-      </x:c>
+        <x:v>wid</x:v>
+      </x:c>
+      <x:c r="G19" s="16" t="str"/>
       <x:c r="H19" s="16" t="str"/>
       <x:c r="I19" s="25" t="str">
-        <x:v>SearchPage._activeQuery；SearchResultItem.entityId</x:v>
+        <x:v>WorldPage.widget.wid</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
       <x:c r="A20" s="24" t="str">
-        <x:v>home_my_worlds_click</x:v>
+        <x:v>search_click</x:v>
       </x:c>
       <x:c r="B20" s="16" t="str">
-        <x:v>点击 My worlds item</x:v>
+        <x:v>点击搜索结果</x:v>
       </x:c>
       <x:c r="C20" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1974,23 +1972,25 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E20" s="16" t="str">
-        <x:v>home_my_worlds_click</x:v>
+        <x:v>search_click</x:v>
       </x:c>
       <x:c r="F20" s="16" t="str">
-        <x:v>wid</x:v>
-      </x:c>
-      <x:c r="G20" s="16" t="str"/>
+        <x:v>query</x:v>
+      </x:c>
+      <x:c r="G20" s="16" t="str">
+        <x:v>oid/wid/uid</x:v>
+      </x:c>
       <x:c r="H20" s="16" t="str"/>
       <x:c r="I20" s="25" t="str">
-        <x:v>WorldListItem.wid</x:v>
+        <x:v>SearchPage._activeQuery；SearchResultItem.entityId</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
       <x:c r="A21" s="24" t="str">
-        <x:v>home_popular_click</x:v>
+        <x:v>home_my_worlds_click</x:v>
       </x:c>
       <x:c r="B21" s="16" t="str">
-        <x:v>点击 Popular item</x:v>
+        <x:v>点击 My worlds item</x:v>
       </x:c>
       <x:c r="C21" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -1999,23 +1999,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E21" s="16" t="str">
-        <x:v>home_popular_click</x:v>
+        <x:v>home_my_worlds_click</x:v>
       </x:c>
       <x:c r="F21" s="16" t="str">
-        <x:v>oid</x:v>
+        <x:v>wid</x:v>
       </x:c>
       <x:c r="G21" s="16" t="str"/>
       <x:c r="H21" s="16" t="str"/>
       <x:c r="I21" s="25" t="str">
-        <x:v>OriginListItem.oid</x:v>
+        <x:v>WorldListItem.wid</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="24" t="str">
-        <x:v>worldo_list_click</x:v>
+        <x:v>home_popular_click</x:v>
       </x:c>
       <x:c r="B22" s="16" t="str">
-        <x:v>点击 worldo list item</x:v>
+        <x:v>点击 Popular item</x:v>
       </x:c>
       <x:c r="C22" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2024,7 +2024,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E22" s="16" t="str">
-        <x:v>worldo_list_click</x:v>
+        <x:v>home_popular_click</x:v>
       </x:c>
       <x:c r="F22" s="16" t="str">
         <x:v>oid</x:v>
@@ -2037,10 +2037,10 @@
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
       <x:c r="A23" s="24" t="str">
-        <x:v>me_click</x:v>
+        <x:v>worldo_list_click</x:v>
       </x:c>
       <x:c r="B23" s="16" t="str">
-        <x:v>点击 Me/Profile 页面 oid/wid 内容</x:v>
+        <x:v>点击 worldo list item</x:v>
       </x:c>
       <x:c r="C23" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2049,23 +2049,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E23" s="16" t="str">
-        <x:v>me_click</x:v>
+        <x:v>worldo_list_click</x:v>
       </x:c>
       <x:c r="F23" s="16" t="str">
-        <x:v>oid/wid</x:v>
+        <x:v>oid</x:v>
       </x:c>
       <x:c r="G23" s="16" t="str"/>
       <x:c r="H23" s="16" t="str"/>
       <x:c r="I23" s="25" t="str">
-        <x:v>UserProfileOriginItem.oid 或 UserProfileWorldItem.wid</x:v>
+        <x:v>OriginListItem.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
       <x:c r="A24" s="24" t="str">
-        <x:v>worldo_map_click</x:v>
+        <x:v>me_click</x:v>
       </x:c>
       <x:c r="B24" s="16" t="str">
-        <x:v>点击旧版 worldo map 任意位置</x:v>
+        <x:v>点击 Me/Profile 页面 oid/wid 内容</x:v>
       </x:c>
       <x:c r="C24" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2074,23 +2074,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E24" s="16" t="str">
-        <x:v>worldo_map_click</x:v>
+        <x:v>me_click</x:v>
       </x:c>
       <x:c r="F24" s="16" t="str">
-        <x:v>oid</x:v>
+        <x:v>oid/wid</x:v>
       </x:c>
       <x:c r="G24" s="16" t="str"/>
       <x:c r="H24" s="16" t="str"/>
       <x:c r="I24" s="25" t="str">
-        <x:v>OriginDetail.oid</x:v>
+        <x:v>UserProfileOriginItem.oid 或 UserProfileWorldItem.wid</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="24" t="str">
-        <x:v>worldo_tilemap_click</x:v>
+        <x:v>worldo_map_click</x:v>
       </x:c>
       <x:c r="B25" s="16" t="str">
-        <x:v>点击 Tilemap 版 worldo map 任意位置</x:v>
+        <x:v>点击旧版 worldo map 任意位置</x:v>
       </x:c>
       <x:c r="C25" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2099,7 +2099,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E25" s="16" t="str">
-        <x:v>worldo_tilemap_click</x:v>
+        <x:v>worldo_map_click</x:v>
       </x:c>
       <x:c r="F25" s="16" t="str">
         <x:v>oid</x:v>
@@ -2112,10 +2112,10 @@
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="24" t="str">
-        <x:v>world_locations_click</x:v>
+        <x:v>worldo_tilemap_click</x:v>
       </x:c>
       <x:c r="B26" s="16" t="str">
-        <x:v>点击 location 列表项</x:v>
+        <x:v>点击 Tilemap 版 worldo map 任意位置</x:v>
       </x:c>
       <x:c r="C26" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2124,25 +2124,23 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E26" s="16" t="str">
-        <x:v>world_locations_click</x:v>
+        <x:v>worldo_tilemap_click</x:v>
       </x:c>
       <x:c r="F26" s="16" t="str">
-        <x:v>wid</x:v>
-      </x:c>
-      <x:c r="G26" s="16" t="str">
-        <x:v>loc_id</x:v>
-      </x:c>
+        <x:v>oid</x:v>
+      </x:c>
+      <x:c r="G26" s="16" t="str"/>
       <x:c r="H26" s="16" t="str"/>
       <x:c r="I26" s="25" t="str">
-        <x:v>WorldDetail.worldId；WorldPoint sceneId/pointId/id</x:v>
+        <x:v>OriginDetail.oid</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
       <x:c r="A27" s="24" t="str">
-        <x:v>world_map_click</x:v>
+        <x:v>world_locations_click</x:v>
       </x:c>
       <x:c r="B27" s="16" t="str">
-        <x:v>点击旧版 world map 任意位置</x:v>
+        <x:v>点击 location 列表项</x:v>
       </x:c>
       <x:c r="C27" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2151,23 +2149,25 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E27" s="16" t="str">
-        <x:v>world_map_click</x:v>
+        <x:v>world_locations_click</x:v>
       </x:c>
       <x:c r="F27" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G27" s="16" t="str"/>
+      <x:c r="G27" s="16" t="str">
+        <x:v>loc_id</x:v>
+      </x:c>
       <x:c r="H27" s="16" t="str"/>
       <x:c r="I27" s="25" t="str">
-        <x:v>WorldPage.widget.wid</x:v>
+        <x:v>WorldDetail.worldId；WorldPoint sceneId/pointId/id</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="30" customHeight="1">
       <x:c r="A28" s="24" t="str">
-        <x:v>world_tilemap_click</x:v>
+        <x:v>world_map_click</x:v>
       </x:c>
       <x:c r="B28" s="16" t="str">
-        <x:v>点击 Tilemap 版 world map 任意位置</x:v>
+        <x:v>点击旧版 world map 任意位置</x:v>
       </x:c>
       <x:c r="C28" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2176,7 +2176,7 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E28" s="16" t="str">
-        <x:v>world_tilemap_click</x:v>
+        <x:v>world_map_click</x:v>
       </x:c>
       <x:c r="F28" s="16" t="str">
         <x:v>wid</x:v>
@@ -2189,10 +2189,10 @@
     </x:row>
     <x:row r="29" ht="30" customHeight="1">
       <x:c r="A29" s="24" t="str">
-        <x:v>location_chat_send_message</x:v>
+        <x:v>world_tilemap_click</x:v>
       </x:c>
       <x:c r="B29" s="16" t="str">
-        <x:v>location chat 发消息成功后</x:v>
+        <x:v>点击 Tilemap 版 world map 任意位置</x:v>
       </x:c>
       <x:c r="C29" s="16" t="str">
         <x:v>GenesisTelemetry.collectLog</x:v>
@@ -2201,52 +2201,77 @@
         <x:v>event</x:v>
       </x:c>
       <x:c r="E29" s="16" t="str">
-        <x:v>location_chat_send_message</x:v>
+        <x:v>world_tilemap_click</x:v>
       </x:c>
       <x:c r="F29" s="16" t="str">
         <x:v>wid</x:v>
       </x:c>
-      <x:c r="G29" s="16" t="str">
+      <x:c r="G29" s="16" t="str"/>
+      <x:c r="H29" s="16" t="str"/>
+      <x:c r="I29" s="25" t="str">
+        <x:v>WorldPage.widget.wid</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="30" customHeight="1">
+      <x:c r="A30" s="24" t="str">
+        <x:v>location_chat_send_message</x:v>
+      </x:c>
+      <x:c r="B30" s="16" t="str">
+        <x:v>location chat 发消息成功后</x:v>
+      </x:c>
+      <x:c r="C30" s="16" t="str">
+        <x:v>GenesisTelemetry.collectLog</x:v>
+      </x:c>
+      <x:c r="D30" s="16" t="str">
+        <x:v>event</x:v>
+      </x:c>
+      <x:c r="E30" s="16" t="str">
+        <x:v>location_chat_send_message</x:v>
+      </x:c>
+      <x:c r="F30" s="16" t="str">
+        <x:v>wid</x:v>
+      </x:c>
+      <x:c r="G30" s="16" t="str">
         <x:v>loc_id</x:v>
       </x:c>
-      <x:c r="H29" s="16" t="str">
+      <x:c r="H30" s="16" t="str">
         <x:v>message_id</x:v>
       </x:c>
-      <x:c r="I29" s="25" t="str">
+      <x:c r="I30" s="25" t="str">
         <x:v>LocationChatPage.widget.worldId；widget.locationId；ack.messageId</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="30" customHeight="1">
-      <x:c r="A30" s="26" t="str">
+    <x:row r="31" ht="30" customHeight="1">
+      <x:c r="A31" s="26" t="str">
         <x:v>private_chat_send_message</x:v>
       </x:c>
-      <x:c r="B30" s="27" t="str">
+      <x:c r="B31" s="27" t="str">
         <x:v>私聊发送成功后</x:v>
       </x:c>
-      <x:c r="C30" s="27" t="str">
-        <x:v>GenesisTelemetry.collectLog</x:v>
-      </x:c>
-      <x:c r="D30" s="27" t="str">
-        <x:v>event</x:v>
-      </x:c>
-      <x:c r="E30" s="27" t="str">
+      <x:c r="C31" s="27" t="str">
+        <x:v>GenesisTelemetry.collectLog</x:v>
+      </x:c>
+      <x:c r="D31" s="27" t="str">
+        <x:v>event</x:v>
+      </x:c>
+      <x:c r="E31" s="27" t="str">
         <x:v>private_chat_send_message</x:v>
       </x:c>
-      <x:c r="F30" s="27" t="str">
+      <x:c r="F31" s="27" t="str">
         <x:v>peer_uid</x:v>
       </x:c>
-      <x:c r="G30" s="27" t="str">
+      <x:c r="G31" s="27" t="str">
         <x:v>message_id</x:v>
       </x:c>
-      <x:c r="H30" s="27" t="str"/>
-      <x:c r="I30" s="28" t="str">
+      <x:c r="H31" s="27" t="str"/>
+      <x:c r="I31" s="28" t="str">
         <x:v>ChatPage._peerUid；dm send 返回 message_id/id</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R731b57d7abd54656"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71ca6502203a403b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>